<commit_message>
Layout of PCB mostly done
</commit_message>
<xml_diff>
--- a/Documentation/Avionics-Electrical-CID-Rev00.xlsx
+++ b/Documentation/Avionics-Electrical-CID-Rev00.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alger\OneDrive\Bureau\RocketPower\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA81FDE3-4D48-4097-B851-733B25FBCBEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06614C33-DC6C-417E-9A51-4F9DD813B4DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{3EEFD8E8-0D7E-45CD-A648-966D5F240C39}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="1" xr2:uid="{3EEFD8E8-0D7E-45CD-A648-966D5F240C39}"/>
   </bookViews>
   <sheets>
     <sheet name="Teensy Interface" sheetId="1" r:id="rId1"/>
-    <sheet name="MCU Interface" sheetId="2" r:id="rId2"/>
+    <sheet name="Components" sheetId="3" r:id="rId2"/>
+    <sheet name="MCU Interface" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="81">
   <si>
     <t>GND</t>
   </si>
@@ -262,6 +263,24 @@
   </si>
   <si>
     <t xml:space="preserve">IMU LED </t>
+  </si>
+  <si>
+    <t>Reserve PWM</t>
+  </si>
+  <si>
+    <t>Components</t>
+  </si>
+  <si>
+    <t>Remove before flight switch</t>
+  </si>
+  <si>
+    <t>https://www.mouser.ca/datasheet/3/39/1/B032-E1.pdf</t>
+  </si>
+  <si>
+    <t>Reset Button</t>
+  </si>
+  <si>
+    <t>https://www.mouser.ca/ProductDetail/CK/KMR241G-LFS?qs=Qe4e1uPWiB0VU4olKDUEuQ%3D%3D&amp;srsltid=AfmBOor8Xhp69zXd1t5T1eV3rP8WAkpNAXf_olLCyJLNUTt_QkTjkPpR</t>
   </si>
 </sst>
 </file>
@@ -732,16 +751,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ADE3831-046D-4225-BB55-A67055906E37}">
   <dimension ref="B6:N30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.5703125" customWidth="1"/>
+    <col min="1" max="1" width="6.5546875" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="13" max="13" width="28.42578125" customWidth="1"/>
-    <col min="14" max="14" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" customWidth="1"/>
+    <col min="13" max="13" width="28.44140625" customWidth="1"/>
+    <col min="14" max="14" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
         <v>13</v>
       </c>
@@ -755,7 +774,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
       <c r="C7" s="1" t="s">
         <v>0</v>
       </c>
@@ -763,7 +782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>8</v>
       </c>
@@ -774,7 +793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>7</v>
       </c>
@@ -785,35 +804,35 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>6</v>
       </c>
       <c r="C10" t="s">
         <v>5</v>
       </c>
-      <c r="M10" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="N10" s="3" t="s">
+      <c r="M10" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="N10" s="5" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>10</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
       </c>
-      <c r="M11" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="N11" s="3" t="s">
+      <c r="M11" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="N11" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>11</v>
       </c>
@@ -827,7 +846,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>15</v>
       </c>
@@ -841,7 +860,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>16</v>
       </c>
@@ -855,7 +874,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>19</v>
       </c>
@@ -869,7 +888,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>22</v>
       </c>
@@ -883,7 +902,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>23</v>
       </c>
@@ -897,7 +916,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>24</v>
       </c>
@@ -911,7 +930,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>25</v>
       </c>
@@ -925,7 +944,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>26</v>
       </c>
@@ -939,7 +958,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
       <c r="C21" s="1" t="s">
         <v>2</v>
       </c>
@@ -947,7 +966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>27</v>
       </c>
@@ -961,7 +980,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>28</v>
       </c>
@@ -975,7 +994,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B24" s="5" t="s">
         <v>29</v>
       </c>
@@ -989,7 +1008,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B25" s="5" t="s">
         <v>30</v>
       </c>
@@ -1003,7 +1022,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>31</v>
       </c>
@@ -1017,7 +1036,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>32</v>
       </c>
@@ -1031,7 +1050,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>33</v>
       </c>
@@ -1045,7 +1064,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>34</v>
       </c>
@@ -1059,7 +1078,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>35</v>
       </c>
@@ -1082,9 +1101,43 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33450D7B-CA85-429F-9414-16B0B8619FF9}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0DC2028-9F9E-4718-82E0-6186DDEF695E}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>